<commit_message>
week 25 update — championship finale dispatch, final odds, keepers refresh
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/LPT-Keeper-Status-2026.xlsx
+++ b/downloads/LPT-Keeper-Status-2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="2027 Keeper Outlook" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2027 Keeper Outlook'!$A$1:$G$526</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2027 Keeper Outlook'!$A$1:$G$525</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G526"/>
+  <dimension ref="A1:G525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -730,16 +730,16 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Robbie Ray</t>
+          <t>Isaac Paredes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -763,12 +763,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Isaac Paredes</t>
+          <t>Cam Schlittler</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Cam Schlittler</t>
+          <t>Carlos Rodón</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -829,12 +829,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Carlos Rodón</t>
+          <t>Abner Uribe</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -862,20 +862,20 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Abner Uribe</t>
+          <t>Coby Mayo</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
@@ -895,12 +895,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>Jared Jones</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
@@ -928,24 +928,24 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Jared Jones</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="16">
@@ -961,24 +961,24 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Nick Kurtz</t>
+          <t>Richie Palacios</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="17">
@@ -1192,16 +1192,16 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Grant Holmes</t>
+          <t>Andrew Alvarez</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>WSN</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Gregory Soto</t>
+          <t>Grant Holmes</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
@@ -1258,12 +1258,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Gregory Soto</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -1291,12 +1291,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -1324,12 +1324,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Davis Martin</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Kevin Kelly</t>
+          <t>Davis Martin</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Leo Bernal</t>
+          <t>Kevin Kelly</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
@@ -1423,12 +1423,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Paul Skenes</t>
+          <t>Leo Bernal</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
@@ -1436,11 +1436,11 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="31">
@@ -1456,12 +1456,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Max Clark</t>
+          <t>Paul Skenes</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
@@ -1469,11 +1469,11 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="32">
@@ -1489,12 +1489,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Andrew Alvarez</t>
+          <t>Max Clark</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="33">
@@ -1555,21 +1555,25 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Richie Palacios</t>
+          <t>Jonah Tong</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr"/>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Unknown (no acquisition record)</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>2028</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3993,24 +3997,24 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Joe Ryan</t>
+          <t>Dustin May</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="109">
@@ -4026,24 +4030,24 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Shane McClanahan</t>
+          <t>Joe Ryan</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="110">
@@ -4059,7 +4063,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Drew Rasmussen</t>
+          <t>Shane McClanahan</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -4068,7 +4072,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4092,16 +4096,16 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Drew Rasmussen</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -4125,12 +4129,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -4158,16 +4162,16 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -4191,12 +4195,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4224,20 +4228,20 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G115" t="n">
@@ -4257,16 +4261,16 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Brendan Donovan</t>
+          <t>Jeff Hoffman</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -4290,24 +4294,24 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Mason Miller</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="118">
@@ -4323,20 +4327,20 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Brendan Donovan</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G118" t="n">
@@ -4356,24 +4360,24 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Gerrit Cole</t>
+          <t>Mason Miller</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="120">
@@ -4389,12 +4393,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Jackson Jobe</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4402,11 +4406,11 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G120" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="121">
@@ -4422,24 +4426,24 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Cal Quantrill</t>
+          <t>Gerrit Cole</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G121" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="122">
@@ -4455,24 +4459,24 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Andrew Painter</t>
+          <t>Jackson Jobe</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G122" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="123">
@@ -4488,12 +4492,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Cal Quantrill</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -4521,16 +4525,16 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Clay Holmes</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -4554,12 +4558,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Adrian Morejon</t>
+          <t>Clay Holmes</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -4567,11 +4571,11 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="126">
@@ -4587,12 +4591,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Garrett Whitlock</t>
+          <t>Adrian Morejon</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4600,7 +4604,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G126" t="n">
@@ -4620,12 +4624,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Garrett Whitlock</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4633,7 +4637,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G127" t="n">
@@ -4653,12 +4657,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Bryan Baker</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -4666,11 +4670,11 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G128" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="129">
@@ -4686,12 +4690,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Heriberto Hernández</t>
+          <t>Bryan Baker</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -4719,12 +4723,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Tim Tawa</t>
+          <t>Bubba Chandler</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -4732,7 +4736,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G130" t="n">
@@ -4752,12 +4756,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Samuel Basallo</t>
+          <t>Heriberto Hernández</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -4765,7 +4769,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (pre-season waiver origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G131" t="n">
@@ -4785,12 +4789,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Kodai Senga</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4818,12 +4822,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Bryan Woo</t>
+          <t>Tim Tawa</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4831,11 +4835,11 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G133" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="134">
@@ -4851,12 +4855,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -4884,12 +4888,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Franklin Arias</t>
+          <t>Bryan Woo</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -4897,11 +4901,11 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="136">
@@ -4917,12 +4921,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Kade Anderson</t>
+          <t>Franklin Arias</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -5940,12 +5944,12 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>Yusei Kikuchi</t>
+          <t>Evan Phillips</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E167" s="2" t="n">
@@ -5953,11 +5957,11 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="168">
@@ -5973,12 +5977,12 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Joshua Baez</t>
+          <t>Yusei Kikuchi</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E168" s="2" t="n">
@@ -5986,7 +5990,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G168" s="2" t="n">
@@ -6006,12 +6010,12 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Joshua Baez</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E169" s="2" t="n">
@@ -6039,12 +6043,12 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E170" s="2" t="n">
@@ -6072,21 +6076,25 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Evan Phillips</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
-        </is>
-      </c>
-      <c r="E171" s="2" t="inlineStr"/>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>Unknown (no acquisition record)</t>
-        </is>
-      </c>
-      <c r="G171" s="2" t="inlineStr"/>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="n">
+        <v>2028</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6398,16 +6406,16 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F181" t="inlineStr">
         <is>
@@ -6431,16 +6439,16 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Willson Contreras</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F182" t="inlineStr">
         <is>
@@ -6464,12 +6472,12 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Willson Contreras</t>
+          <t>Emmet Sheehan</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -6497,24 +6505,24 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Emmet Sheehan</t>
+          <t>Jacob deGrom</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G184" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="185">
@@ -6530,12 +6538,12 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Jacob deGrom</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -6543,11 +6551,11 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G185" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="186">
@@ -6563,12 +6571,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Ryan Johnson</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -6576,11 +6584,11 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G186" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="187">
@@ -6596,24 +6604,24 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G187" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="188">
@@ -6629,24 +6637,24 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Kyle Stowers</t>
+          <t>Tanner Scott</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G188" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="189">
@@ -6662,16 +6670,16 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Quinn Mathews</t>
+          <t>Tyler Wells</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F189" t="inlineStr">
         <is>
@@ -6695,12 +6703,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Tanner Scott</t>
+          <t>Cade Smith</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -6708,11 +6716,11 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G190" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="191">
@@ -6728,12 +6736,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Tyler Wells</t>
+          <t>Andrew Painter</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -6741,11 +6749,11 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G191" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="192">
@@ -6761,12 +6769,12 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Cade Smith</t>
+          <t>River Ryan</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -6774,11 +6782,11 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G192" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="193">
@@ -6794,24 +6802,24 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>River Ryan</t>
+          <t>Bryan Hudson</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G193" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="194">
@@ -6827,12 +6835,12 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Louis Varland</t>
+          <t>Luis Medina</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -6860,7 +6868,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Brent Headrick</t>
+          <t>Anthony Volpe</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -6873,11 +6881,11 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G195" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="196">
@@ -6893,12 +6901,12 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Louis Varland</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E196" t="n">
@@ -6906,7 +6914,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G196" t="n">
@@ -6926,12 +6934,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Brent Headrick</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E197" t="n">
@@ -6939,11 +6947,11 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G197" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="198">
@@ -6959,12 +6967,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -6972,11 +6980,11 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G198" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="199">
@@ -6992,12 +7000,12 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Troy Melton</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E199" t="n">
@@ -7005,11 +7013,11 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G199" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="200">
@@ -7025,12 +7033,12 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -7038,11 +7046,11 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G200" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="201">
@@ -7058,12 +7066,12 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Mason Montgomery</t>
+          <t>Spencer Jones</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E201" t="n">
@@ -7091,12 +7099,12 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Junior Caminero</t>
+          <t>Mason Montgomery</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -7104,11 +7112,11 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G202" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="203">
@@ -7124,12 +7132,12 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Charlie Condon</t>
+          <t>Junior Caminero</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -7137,11 +7145,11 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G203" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="204">
@@ -7157,12 +7165,12 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Bradgley Rodriguez</t>
+          <t>Quinn Mathews</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E204" t="n">
@@ -7190,21 +7198,25 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Bryan Hudson</t>
+          <t>Bradgley Rodriguez</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>CWS</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr"/>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>1</v>
+      </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Unknown (no acquisition record)</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr"/>
+          <t>Waiver — year 1 of 2</t>
+        </is>
+      </c>
+      <c r="G205" t="n">
+        <v>2027</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -10322,7 +10334,7 @@
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E300" s="2" t="n">
@@ -11147,7 +11159,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E325" t="n">
@@ -14112,24 +14124,24 @@
       </c>
       <c r="C415" s="3" t="inlineStr">
         <is>
-          <t>Hunter Greene</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="D415" s="3" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E415" s="3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F415" s="3" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G415" s="3" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="416">
@@ -14145,24 +14157,24 @@
       </c>
       <c r="C416" s="3" t="inlineStr">
         <is>
-          <t>Ryan Pepiot</t>
+          <t>Hunter Greene</t>
         </is>
       </c>
       <c r="D416" s="3" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="E416" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F416" s="3" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
+          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
         </is>
       </c>
       <c r="G416" s="3" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="417">
@@ -14178,12 +14190,12 @@
       </c>
       <c r="C417" s="3" t="inlineStr">
         <is>
-          <t>Noelvi Marte</t>
+          <t>Ryan Pepiot</t>
         </is>
       </c>
       <c r="D417" s="3" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>TBR</t>
         </is>
       </c>
       <c r="E417" s="3" t="n">
@@ -14211,16 +14223,16 @@
       </c>
       <c r="C418" s="3" t="inlineStr">
         <is>
-          <t>Cade Horton</t>
+          <t>Noelvi Marte</t>
         </is>
       </c>
       <c r="D418" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="E418" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F418" s="3" t="inlineStr">
         <is>
@@ -14244,12 +14256,12 @@
       </c>
       <c r="C419" s="3" t="inlineStr">
         <is>
-          <t>Luis Castillo</t>
+          <t>Cade Horton</t>
         </is>
       </c>
       <c r="D419" s="3" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E419" s="3" t="n">
@@ -14277,7 +14289,7 @@
       </c>
       <c r="C420" s="3" t="inlineStr">
         <is>
-          <t>Brenton Doyle</t>
+          <t>Luis Castillo</t>
         </is>
       </c>
       <c r="D420" s="3" t="inlineStr">
@@ -14286,7 +14298,7 @@
         </is>
       </c>
       <c r="E420" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F420" s="3" t="inlineStr">
         <is>
@@ -14310,12 +14322,12 @@
       </c>
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Brenton Doyle</t>
         </is>
       </c>
       <c r="D421" s="3" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E421" s="3" t="n">
@@ -14343,12 +14355,12 @@
       </c>
       <c r="C422" s="3" t="inlineStr">
         <is>
-          <t>Spencer Strider</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="D422" s="3" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E422" s="3" t="n">
@@ -14376,12 +14388,12 @@
       </c>
       <c r="C423" s="3" t="inlineStr">
         <is>
-          <t>Jordan Lawlar</t>
+          <t>Spencer Strider</t>
         </is>
       </c>
       <c r="D423" s="3" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E423" s="3" t="n">
@@ -14389,7 +14401,7 @@
       </c>
       <c r="F423" s="3" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G423" s="3" t="n">
@@ -14409,24 +14421,24 @@
       </c>
       <c r="C424" s="3" t="inlineStr">
         <is>
-          <t>Josh Lowe</t>
+          <t>Jordan Lawlar</t>
         </is>
       </c>
       <c r="D424" s="3" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E424" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F424" s="3" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
         </is>
       </c>
       <c r="G424" s="3" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="425">
@@ -14442,12 +14454,12 @@
       </c>
       <c r="C425" s="3" t="inlineStr">
         <is>
-          <t>Jeff Hoffman</t>
+          <t>Josh Lowe</t>
         </is>
       </c>
       <c r="D425" s="3" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E425" s="3" t="n">
@@ -14455,11 +14467,11 @@
       </c>
       <c r="F425" s="3" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
+          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
         </is>
       </c>
       <c r="G425" s="3" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="426">
@@ -14541,16 +14553,16 @@
       </c>
       <c r="C428" s="3" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Robbie Ray</t>
         </is>
       </c>
       <c r="D428" s="3" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E428" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F428" s="3" t="inlineStr">
         <is>
@@ -14574,12 +14586,12 @@
       </c>
       <c r="C429" s="3" t="inlineStr">
         <is>
-          <t>Carlos Estévez</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="D429" s="3" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E429" s="3" t="n">
@@ -14607,12 +14619,12 @@
       </c>
       <c r="C430" s="3" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Carlos Estévez</t>
         </is>
       </c>
       <c r="D430" s="3" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>KCR</t>
         </is>
       </c>
       <c r="E430" s="3" t="n">
@@ -14640,16 +14652,16 @@
       </c>
       <c r="C431" s="3" t="inlineStr">
         <is>
-          <t>Edward Cabrera</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="D431" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E431" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F431" s="3" t="inlineStr">
         <is>
@@ -14673,12 +14685,12 @@
       </c>
       <c r="C432" s="3" t="inlineStr">
         <is>
-          <t>Pete Fairbanks</t>
+          <t>Edward Cabrera</t>
         </is>
       </c>
       <c r="D432" s="3" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E432" s="3" t="n">
@@ -14706,24 +14718,24 @@
       </c>
       <c r="C433" s="3" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Pete Fairbanks</t>
         </is>
       </c>
       <c r="D433" s="3" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E433" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F433" s="3" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin); MAXED OUT — cannot be kept if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G433" s="3" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="434">
@@ -14739,12 +14751,12 @@
       </c>
       <c r="C434" s="3" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="D434" s="3" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E434" s="3" t="n">
@@ -14772,12 +14784,12 @@
       </c>
       <c r="C435" s="3" t="inlineStr">
         <is>
-          <t>Tatsuya Imai</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="D435" s="3" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E435" s="3" t="n">
@@ -14785,11 +14797,11 @@
       </c>
       <c r="F435" s="3" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
+          <t>Kept — final year (draft origin); MAXED OUT — cannot be kept if re-added</t>
         </is>
       </c>
       <c r="G435" s="3" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="436">
@@ -14805,12 +14817,12 @@
       </c>
       <c r="C436" s="3" t="inlineStr">
         <is>
-          <t>TJ Friedl</t>
+          <t>Tatsuya Imai</t>
         </is>
       </c>
       <c r="D436" s="3" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="E436" s="3" t="n">
@@ -14838,12 +14850,12 @@
       </c>
       <c r="C437" s="3" t="inlineStr">
         <is>
-          <t>Sal Frelick</t>
+          <t>TJ Friedl</t>
         </is>
       </c>
       <c r="D437" s="3" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="E437" s="3" t="n">
@@ -14871,12 +14883,12 @@
       </c>
       <c r="C438" s="3" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Sal Frelick</t>
         </is>
       </c>
       <c r="D438" s="3" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E438" s="3" t="n">
@@ -14904,12 +14916,12 @@
       </c>
       <c r="C439" s="3" t="inlineStr">
         <is>
-          <t>Kyle Teel</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="D439" s="3" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E439" s="3" t="n">
@@ -14937,12 +14949,12 @@
       </c>
       <c r="C440" s="3" t="inlineStr">
         <is>
-          <t>Connelly Early</t>
+          <t>Kyle Teel</t>
         </is>
       </c>
       <c r="D440" s="3" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E440" s="3" t="n">
@@ -14970,12 +14982,12 @@
       </c>
       <c r="C441" s="3" t="inlineStr">
         <is>
-          <t>Moisés Ballesteros</t>
+          <t>Connelly Early</t>
         </is>
       </c>
       <c r="D441" s="3" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E441" s="3" t="n">
@@ -14983,7 +14995,7 @@
       </c>
       <c r="F441" s="3" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G441" s="3" t="n">
@@ -15003,12 +15015,12 @@
       </c>
       <c r="C442" s="3" t="inlineStr">
         <is>
-          <t>Dylan Beavers</t>
+          <t>Moisés Ballesteros</t>
         </is>
       </c>
       <c r="D442" s="3" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E442" s="3" t="n">
@@ -15036,20 +15048,20 @@
       </c>
       <c r="C443" s="3" t="inlineStr">
         <is>
-          <t>Ramón Laureano</t>
+          <t>Dylan Beavers</t>
         </is>
       </c>
       <c r="D443" s="3" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E443" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F443" s="3" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
         </is>
       </c>
       <c r="G443" s="3" t="n">
@@ -15069,12 +15081,12 @@
       </c>
       <c r="C444" s="3" t="inlineStr">
         <is>
-          <t>Adolis García</t>
+          <t>Ramón Laureano</t>
         </is>
       </c>
       <c r="D444" s="3" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E444" s="3" t="n">
@@ -15102,12 +15114,12 @@
       </c>
       <c r="C445" s="3" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Adolis García</t>
         </is>
       </c>
       <c r="D445" s="3" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E445" s="3" t="n">
@@ -15135,12 +15147,12 @@
       </c>
       <c r="C446" s="3" t="inlineStr">
         <is>
-          <t>Justin Crawford</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="D446" s="3" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E446" s="3" t="n">
@@ -15168,12 +15180,12 @@
       </c>
       <c r="C447" s="3" t="inlineStr">
         <is>
-          <t>Hunter Gaddis</t>
+          <t>Justin Crawford</t>
         </is>
       </c>
       <c r="D447" s="3" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E447" s="3" t="n">
@@ -15181,7 +15193,7 @@
       </c>
       <c r="F447" s="3" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G447" s="3" t="n">
@@ -15201,12 +15213,12 @@
       </c>
       <c r="C448" s="3" t="inlineStr">
         <is>
-          <t>Brendon Little</t>
+          <t>Hunter Gaddis</t>
         </is>
       </c>
       <c r="D448" s="3" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E448" s="3" t="n">
@@ -15234,24 +15246,24 @@
       </c>
       <c r="C449" s="3" t="inlineStr">
         <is>
-          <t>Agustín Ramírez</t>
+          <t>Brendon Little</t>
         </is>
       </c>
       <c r="D449" s="3" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E449" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F449" s="3" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin); MAXED OUT — cannot be kept if re-added</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
         </is>
       </c>
       <c r="G449" s="3" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="450">
@@ -15267,12 +15279,12 @@
       </c>
       <c r="C450" s="3" t="inlineStr">
         <is>
-          <t>Jorge Polanco</t>
+          <t>Agustín Ramírez</t>
         </is>
       </c>
       <c r="D450" s="3" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E450" s="3" t="n">
@@ -15300,12 +15312,12 @@
       </c>
       <c r="C451" s="3" t="inlineStr">
         <is>
-          <t>Zac Gallen</t>
+          <t>Jorge Polanco</t>
         </is>
       </c>
       <c r="D451" s="3" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E451" s="3" t="n">
@@ -15313,11 +15325,11 @@
       </c>
       <c r="F451" s="3" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
+          <t>Kept — final year (waiver origin); MAXED OUT — cannot be kept if re-added</t>
         </is>
       </c>
       <c r="G451" s="3" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="452">
@@ -15333,12 +15345,12 @@
       </c>
       <c r="C452" s="3" t="inlineStr">
         <is>
-          <t>Jordan Westburg</t>
+          <t>Zac Gallen</t>
         </is>
       </c>
       <c r="D452" s="3" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E452" s="3" t="n">
@@ -15366,12 +15378,12 @@
       </c>
       <c r="C453" s="3" t="inlineStr">
         <is>
-          <t>Dennis Santana</t>
+          <t>Jordan Westburg</t>
         </is>
       </c>
       <c r="D453" s="3" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E453" s="3" t="n">
@@ -15399,7 +15411,7 @@
       </c>
       <c r="C454" s="3" t="inlineStr">
         <is>
-          <t>Ryne Nelson</t>
+          <t>Dennis Santana</t>
         </is>
       </c>
       <c r="D454" s="3" t="inlineStr">
@@ -15432,12 +15444,12 @@
       </c>
       <c r="C455" s="3" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Ryne Nelson</t>
         </is>
       </c>
       <c r="D455" s="3" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E455" s="3" t="n">
@@ -15465,12 +15477,12 @@
       </c>
       <c r="C456" s="3" t="inlineStr">
         <is>
-          <t>Edwin Uceta</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="D456" s="3" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E456" s="3" t="n">
@@ -15498,12 +15510,12 @@
       </c>
       <c r="C457" s="3" t="inlineStr">
         <is>
-          <t>Jordan Beck</t>
+          <t>Edwin Uceta</t>
         </is>
       </c>
       <c r="D457" s="3" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>TBR</t>
         </is>
       </c>
       <c r="E457" s="3" t="n">
@@ -15531,12 +15543,12 @@
       </c>
       <c r="C458" s="3" t="inlineStr">
         <is>
-          <t>Jonathan India</t>
+          <t>Jordan Beck</t>
         </is>
       </c>
       <c r="D458" s="3" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E458" s="3" t="n">
@@ -15544,7 +15556,7 @@
       </c>
       <c r="F458" s="3" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G458" s="3" t="n">
@@ -15564,12 +15576,12 @@
       </c>
       <c r="C459" s="3" t="inlineStr">
         <is>
-          <t>Zack Littell</t>
+          <t>Jonathan India</t>
         </is>
       </c>
       <c r="D459" s="3" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>KCR</t>
         </is>
       </c>
       <c r="E459" s="3" t="n">
@@ -15597,12 +15609,12 @@
       </c>
       <c r="C460" s="3" t="inlineStr">
         <is>
-          <t>Jameson Taillon</t>
+          <t>Zack Littell</t>
         </is>
       </c>
       <c r="D460" s="3" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E460" s="3" t="n">
@@ -15630,12 +15642,12 @@
       </c>
       <c r="C461" s="3" t="inlineStr">
         <is>
-          <t>Jack Leiter</t>
+          <t>Jameson Taillon</t>
         </is>
       </c>
       <c r="D461" s="3" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E461" s="3" t="n">
@@ -15663,12 +15675,12 @@
       </c>
       <c r="C462" s="3" t="inlineStr">
         <is>
-          <t>Hyeseong Kim</t>
+          <t>Jack Leiter</t>
         </is>
       </c>
       <c r="D462" s="3" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E462" s="3" t="n">
@@ -15696,24 +15708,24 @@
       </c>
       <c r="C463" s="3" t="inlineStr">
         <is>
-          <t>Daniel Palencia</t>
+          <t>Hyeseong Kim</t>
         </is>
       </c>
       <c r="D463" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E463" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F463" s="3" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin); MAXED OUT — cannot be kept if re-added</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
         </is>
       </c>
       <c r="G463" s="3" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="464">
@@ -15729,12 +15741,12 @@
       </c>
       <c r="C464" s="3" t="inlineStr">
         <is>
-          <t>Jordan Romano</t>
+          <t>Daniel Palencia</t>
         </is>
       </c>
       <c r="D464" s="3" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E464" s="3" t="n">
@@ -15742,11 +15754,11 @@
       </c>
       <c r="F464" s="3" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
+          <t>Kept — final year (waiver origin); MAXED OUT — cannot be kept if re-added</t>
         </is>
       </c>
       <c r="G464" s="3" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="465">
@@ -15762,12 +15774,12 @@
       </c>
       <c r="C465" s="3" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Jordan Romano</t>
         </is>
       </c>
       <c r="D465" s="3" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E465" s="3" t="n">
@@ -15775,11 +15787,11 @@
       </c>
       <c r="F465" s="3" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
+          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
         </is>
       </c>
       <c r="G465" s="3" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="466">
@@ -15795,12 +15807,12 @@
       </c>
       <c r="C466" s="3" t="inlineStr">
         <is>
-          <t>Nolan Schanuel</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="D466" s="3" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="E466" s="3" t="n">
@@ -15828,12 +15840,12 @@
       </c>
       <c r="C467" s="3" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>Nolan Schanuel</t>
         </is>
       </c>
       <c r="D467" s="3" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E467" s="3" t="n">
@@ -15861,12 +15873,12 @@
       </c>
       <c r="C468" s="3" t="inlineStr">
         <is>
-          <t>Quinn Priester</t>
+          <t>Colt Keith</t>
         </is>
       </c>
       <c r="D468" s="3" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E468" s="3" t="n">
@@ -15894,12 +15906,12 @@
       </c>
       <c r="C469" s="3" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Quinn Priester</t>
         </is>
       </c>
       <c r="D469" s="3" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E469" s="3" t="n">
@@ -15927,12 +15939,12 @@
       </c>
       <c r="C470" s="3" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="D470" s="3" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E470" s="3" t="n">
@@ -15940,7 +15952,7 @@
       </c>
       <c r="F470" s="3" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G470" s="3" t="n">
@@ -15960,12 +15972,12 @@
       </c>
       <c r="C471" s="3" t="inlineStr">
         <is>
-          <t>Dylan Lee</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="D471" s="3" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E471" s="3" t="n">
@@ -15993,12 +16005,12 @@
       </c>
       <c r="C472" s="3" t="inlineStr">
         <is>
-          <t>JoJo Romero</t>
+          <t>Dylan Lee</t>
         </is>
       </c>
       <c r="D472" s="3" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E472" s="3" t="n">
@@ -16026,12 +16038,12 @@
       </c>
       <c r="C473" s="3" t="inlineStr">
         <is>
-          <t>Josh Smith</t>
+          <t>JoJo Romero</t>
         </is>
       </c>
       <c r="D473" s="3" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E473" s="3" t="n">
@@ -16059,24 +16071,24 @@
       </c>
       <c r="C474" s="3" t="inlineStr">
         <is>
-          <t>Bubba Chandler</t>
+          <t>Josh Smith</t>
         </is>
       </c>
       <c r="D474" s="3" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E474" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F474" s="3" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
         </is>
       </c>
       <c r="G474" s="3" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="475">
@@ -16092,12 +16104,12 @@
       </c>
       <c r="C475" s="3" t="inlineStr">
         <is>
-          <t>Jacob Wilson</t>
+          <t>Samuel Basallo</t>
         </is>
       </c>
       <c r="D475" s="3" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E475" s="3" t="n">
@@ -16125,12 +16137,12 @@
       </c>
       <c r="C476" s="3" t="inlineStr">
         <is>
-          <t>Blake Treinen</t>
+          <t>Jacob Wilson</t>
         </is>
       </c>
       <c r="D476" s="3" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E476" s="3" t="n">
@@ -16158,12 +16170,12 @@
       </c>
       <c r="C477" s="3" t="inlineStr">
         <is>
-          <t>Brayan Bello</t>
+          <t>Blake Treinen</t>
         </is>
       </c>
       <c r="D477" s="3" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E477" s="3" t="n">
@@ -16171,7 +16183,7 @@
       </c>
       <c r="F477" s="3" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
+          <t>Kept — year 2 of 3 (pre-season waiver origin); status persists if re-added</t>
         </is>
       </c>
       <c r="G477" s="3" t="n">
@@ -16191,12 +16203,12 @@
       </c>
       <c r="C478" s="3" t="inlineStr">
         <is>
-          <t>Eury Pérez</t>
+          <t>Brayan Bello</t>
         </is>
       </c>
       <c r="D478" s="3" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E478" s="3" t="n">
@@ -16204,7 +16216,7 @@
       </c>
       <c r="F478" s="3" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (pre-season waiver origin); status persists if re-added</t>
+          <t>Kept — year 2 of 3 (draft origin); status persists if re-added</t>
         </is>
       </c>
       <c r="G478" s="3" t="n">
@@ -16224,12 +16236,12 @@
       </c>
       <c r="C479" s="3" t="inlineStr">
         <is>
-          <t>Grayson Rodriguez</t>
+          <t>Eury Pérez</t>
         </is>
       </c>
       <c r="D479" s="3" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E479" s="3" t="n">
@@ -16237,11 +16249,11 @@
       </c>
       <c r="F479" s="3" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
+          <t>Kept — year 2 of 3 (pre-season waiver origin); status persists if re-added</t>
         </is>
       </c>
       <c r="G479" s="3" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="480">
@@ -16257,12 +16269,12 @@
       </c>
       <c r="C480" s="3" t="inlineStr">
         <is>
-          <t>Matt Shaw</t>
+          <t>Grayson Rodriguez</t>
         </is>
       </c>
       <c r="D480" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E480" s="3" t="n">
@@ -16290,12 +16302,12 @@
       </c>
       <c r="C481" s="3" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Matt Shaw</t>
         </is>
       </c>
       <c r="D481" s="3" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E481" s="3" t="n">
@@ -16323,12 +16335,12 @@
       </c>
       <c r="C482" s="3" t="inlineStr">
         <is>
-          <t>Shane Smith</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="D482" s="3" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E482" s="3" t="n">
@@ -16356,12 +16368,12 @@
       </c>
       <c r="C483" s="3" t="inlineStr">
         <is>
-          <t>Mitch Keller</t>
+          <t>Shane Smith</t>
         </is>
       </c>
       <c r="D483" s="3" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>CHW</t>
         </is>
       </c>
       <c r="E483" s="3" t="n">
@@ -16389,12 +16401,12 @@
       </c>
       <c r="C484" s="3" t="inlineStr">
         <is>
-          <t>Reynaldo López</t>
+          <t>Mitch Keller</t>
         </is>
       </c>
       <c r="D484" s="3" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E484" s="3" t="n">
@@ -16422,12 +16434,12 @@
       </c>
       <c r="C485" s="3" t="inlineStr">
         <is>
-          <t>Chad Patrick</t>
+          <t>Reynaldo López</t>
         </is>
       </c>
       <c r="D485" s="3" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E485" s="3" t="n">
@@ -16455,12 +16467,12 @@
       </c>
       <c r="C486" s="3" t="inlineStr">
         <is>
-          <t>Giancarlo Stanton</t>
+          <t>Chad Patrick</t>
         </is>
       </c>
       <c r="D486" s="3" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E486" s="3" t="n">
@@ -16488,12 +16500,12 @@
       </c>
       <c r="C487" s="3" t="inlineStr">
         <is>
-          <t>A.J. Minter</t>
+          <t>Giancarlo Stanton</t>
         </is>
       </c>
       <c r="D487" s="3" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E487" s="3" t="n">
@@ -16521,12 +16533,12 @@
       </c>
       <c r="C488" s="3" t="inlineStr">
         <is>
-          <t>Jake Cronenworth</t>
+          <t>A.J. Minter</t>
         </is>
       </c>
       <c r="D488" s="3" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E488" s="3" t="n">
@@ -16554,12 +16566,12 @@
       </c>
       <c r="C489" s="3" t="inlineStr">
         <is>
-          <t>David Peterson</t>
+          <t>Jake Cronenworth</t>
         </is>
       </c>
       <c r="D489" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E489" s="3" t="n">
@@ -16587,12 +16599,12 @@
       </c>
       <c r="C490" s="3" t="inlineStr">
         <is>
-          <t>Jake Mangum</t>
+          <t>David Peterson</t>
         </is>
       </c>
       <c r="D490" s="3" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E490" s="3" t="n">
@@ -16620,12 +16632,12 @@
       </c>
       <c r="C491" s="3" t="inlineStr">
         <is>
-          <t>Ryan Weathers</t>
+          <t>Jake Mangum</t>
         </is>
       </c>
       <c r="D491" s="3" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E491" s="3" t="n">
@@ -16653,12 +16665,12 @@
       </c>
       <c r="C492" s="3" t="inlineStr">
         <is>
-          <t>Garrett Cleavinger</t>
+          <t>Ryan Weathers</t>
         </is>
       </c>
       <c r="D492" s="3" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E492" s="3" t="n">
@@ -16686,12 +16698,12 @@
       </c>
       <c r="C493" s="3" t="inlineStr">
         <is>
-          <t>Matt Brash</t>
+          <t>Garrett Cleavinger</t>
         </is>
       </c>
       <c r="D493" s="3" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E493" s="3" t="n">
@@ -16719,12 +16731,12 @@
       </c>
       <c r="C494" s="3" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Matt Brash</t>
         </is>
       </c>
       <c r="D494" s="3" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E494" s="3" t="n">
@@ -16752,12 +16764,12 @@
       </c>
       <c r="C495" s="3" t="inlineStr">
         <is>
-          <t>Mike Burrows</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="D495" s="3" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E495" s="3" t="n">
@@ -16785,12 +16797,12 @@
       </c>
       <c r="C496" s="3" t="inlineStr">
         <is>
-          <t>Gabe Speier</t>
+          <t>Mike Burrows</t>
         </is>
       </c>
       <c r="D496" s="3" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="E496" s="3" t="n">
@@ -16818,12 +16830,12 @@
       </c>
       <c r="C497" s="3" t="inlineStr">
         <is>
-          <t>Corbin Burnes</t>
+          <t>Gabe Speier</t>
         </is>
       </c>
       <c r="D497" s="3" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E497" s="3" t="n">
@@ -16831,7 +16843,7 @@
       </c>
       <c r="F497" s="3" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
+          <t>Drafted 2026 — year 1 of 3; status persists if re-added</t>
         </is>
       </c>
       <c r="G497" s="3" t="n">
@@ -16851,12 +16863,12 @@
       </c>
       <c r="C498" s="3" t="inlineStr">
         <is>
-          <t>Anthony Volpe</t>
+          <t>Corbin Burnes</t>
         </is>
       </c>
       <c r="D498" s="3" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E498" s="3" t="n">
@@ -17346,12 +17358,12 @@
       </c>
       <c r="C513" s="3" t="inlineStr">
         <is>
-          <t>Jonah Tong</t>
+          <t>Phil Maton</t>
         </is>
       </c>
       <c r="D513" s="3" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E513" s="3" t="n">
@@ -17379,12 +17391,12 @@
       </c>
       <c r="C514" s="3" t="inlineStr">
         <is>
-          <t>Phil Maton</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="D514" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E514" s="3" t="n">
@@ -17412,12 +17424,12 @@
       </c>
       <c r="C515" s="3" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Mick Abel</t>
         </is>
       </c>
       <c r="D515" s="3" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E515" s="3" t="n">
@@ -17445,12 +17457,12 @@
       </c>
       <c r="C516" s="3" t="inlineStr">
         <is>
-          <t>Mick Abel</t>
+          <t>Max Meyer</t>
         </is>
       </c>
       <c r="D516" s="3" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E516" s="3" t="n">
@@ -17478,12 +17490,12 @@
       </c>
       <c r="C517" s="3" t="inlineStr">
         <is>
-          <t>Max Meyer</t>
+          <t>Hunter Harvey</t>
         </is>
       </c>
       <c r="D517" s="3" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E517" s="3" t="n">
@@ -17511,12 +17523,12 @@
       </c>
       <c r="C518" s="3" t="inlineStr">
         <is>
-          <t>Hunter Harvey</t>
+          <t>Carlos Lagrange</t>
         </is>
       </c>
       <c r="D518" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E518" s="3" t="n">
@@ -17544,12 +17556,12 @@
       </c>
       <c r="C519" s="3" t="inlineStr">
         <is>
-          <t>Carlos Lagrange</t>
+          <t>Jorge Soler</t>
         </is>
       </c>
       <c r="D519" s="3" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E519" s="3" t="n">
@@ -17577,12 +17589,12 @@
       </c>
       <c r="C520" s="3" t="inlineStr">
         <is>
-          <t>Jorge Soler</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="D520" s="3" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E520" s="3" t="n">
@@ -17610,12 +17622,12 @@
       </c>
       <c r="C521" s="3" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Will Vest</t>
         </is>
       </c>
       <c r="D521" s="3" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E521" s="3" t="n">
@@ -17643,12 +17655,12 @@
       </c>
       <c r="C522" s="3" t="inlineStr">
         <is>
-          <t>Will Vest</t>
+          <t>Lenyn Sosa</t>
         </is>
       </c>
       <c r="D522" s="3" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E522" s="3" t="n">
@@ -17676,12 +17688,12 @@
       </c>
       <c r="C523" s="3" t="inlineStr">
         <is>
-          <t>Lenyn Sosa</t>
+          <t>Alexis Díaz</t>
         </is>
       </c>
       <c r="D523" s="3" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E523" s="3" t="n">
@@ -17709,12 +17721,12 @@
       </c>
       <c r="C524" s="3" t="inlineStr">
         <is>
-          <t>Alexis Díaz</t>
+          <t>Victor Scott II</t>
         </is>
       </c>
       <c r="D524" s="3" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E524" s="3" t="n">
@@ -17742,12 +17754,12 @@
       </c>
       <c r="C525" s="3" t="inlineStr">
         <is>
-          <t>Victor Scott II</t>
+          <t>Clayton Beeter</t>
         </is>
       </c>
       <c r="D525" s="3" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E525" s="3" t="n">
@@ -17762,41 +17774,8 @@
         <v>2028</v>
       </c>
     </row>
-    <row r="526">
-      <c r="A526" s="3" t="inlineStr">
-        <is>
-          <t>Free Agent</t>
-        </is>
-      </c>
-      <c r="B526" s="3" t="inlineStr">
-        <is>
-          <t>Free Agent</t>
-        </is>
-      </c>
-      <c r="C526" s="3" t="inlineStr">
-        <is>
-          <t>Clayton Beeter</t>
-        </is>
-      </c>
-      <c r="D526" s="3" t="inlineStr">
-        <is>
-          <t>WSH</t>
-        </is>
-      </c>
-      <c r="E526" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F526" s="3" t="inlineStr">
-        <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent); status persists if re-added</t>
-        </is>
-      </c>
-      <c r="G526" s="3" t="n">
-        <v>2028</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G526"/>
+  <autoFilter ref="A1:G525"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
keepers: waiver pickups made after the Aug 6 trade deadline are not keeper-eligible (47 players); transaction log repaired
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/LPT-Keeper-Status-2026.xlsx
+++ b/downloads/LPT-Keeper-Status-2026.xlsx
@@ -961,12 +961,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Richie Palacios</t>
+          <t>Hunter Goodman</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -974,7 +974,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
@@ -994,12 +994,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -1007,11 +1007,11 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="18">
@@ -1027,12 +1027,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Adael Amador</t>
+          <t>C. Encarnacion-Strand</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -1060,12 +1060,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
@@ -1073,11 +1073,11 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="20">
@@ -1093,16 +1093,16 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>C. Encarnacion-Strand</t>
+          <t>Grant Holmes</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1126,16 +1126,16 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Dalton Rushing</t>
+          <t>Gregory Soto</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1159,16 +1159,16 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Erik Sabrowski</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1192,16 +1192,16 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Andrew Alvarez</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Grant Holmes</t>
+          <t>Davis Martin</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
@@ -1258,12 +1258,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Gregory Soto</t>
+          <t>Kevin Kelly</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -1291,12 +1291,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Paul Skenes</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -1304,11 +1304,11 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="27">
@@ -1324,12 +1324,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Max Clark</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
@@ -1337,11 +1337,11 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="28">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Davis Martin</t>
+          <t>Leo De Vries</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
@@ -1370,11 +1370,11 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="29">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Kevin Kelly</t>
+          <t>Jonah Tong</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
@@ -1403,11 +1403,11 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="30">
@@ -1423,25 +1423,21 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Leo Bernal</t>
+          <t>Richie Palacios</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1456,25 +1452,21 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Paul Skenes</t>
+          <t>Adael Amador</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>PIT</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>2026</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1489,25 +1481,21 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Max Clark</t>
+          <t>Leo Bernal</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1522,25 +1510,21 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Leo De Vries</t>
+          <t>Erik Sabrowski</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>ATH</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1555,25 +1539,21 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Jonah Tong</t>
+          <t>Andrew Alvarez</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>NYM</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>WSN</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1951,12 +1931,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Foster Griffin</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -1964,11 +1944,11 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="47">
@@ -1984,24 +1964,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="48">
@@ -2017,24 +1997,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Zebby Matthews</t>
+          <t>Chandler Simpson</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="49">
@@ -2050,24 +2030,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Logan Henderson</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="50">
@@ -2083,24 +2063,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Chandler Simpson</t>
+          <t>Yoendrys Gómez</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="51">
@@ -2116,24 +2096,24 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Martín Pérez</t>
+          <t>Kyle Harrison</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="52">
@@ -2149,7 +2129,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Logan Henderson</t>
+          <t>Jacob Misiorowski</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2158,15 +2138,15 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G52" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="53">
@@ -2182,24 +2162,24 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Zach Thornton</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G53" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="54">
@@ -2215,12 +2195,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Sean Murphy</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -2228,11 +2208,11 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G54" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="55">
@@ -2248,7 +2228,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yoendrys Gómez</t>
+          <t>Kaelen Culpepper</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2281,12 +2261,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Kyle Harrison</t>
+          <t>Brandon Young</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -2294,11 +2274,11 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="57">
@@ -2314,25 +2294,21 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Joey Ortiz</t>
+          <t>Martín Pérez</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>MIL</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>1</v>
-      </c>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2347,25 +2323,21 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Jacob Misiorowski</t>
+          <t>Foster Griffin</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>MIL</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>1</v>
-      </c>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>2026</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2380,25 +2352,21 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Thomas Saggese</t>
+          <t>Sean Murphy</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>STL</t>
-        </is>
-      </c>
-      <c r="E59" t="n">
-        <v>1</v>
-      </c>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G59" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2413,25 +2381,21 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Mickey Gasper</t>
+          <t>Joey Ortiz</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>BOS</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>1</v>
-      </c>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2446,25 +2410,21 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Jacob Lopez</t>
+          <t>Thomas Saggese</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ATH</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>1</v>
-      </c>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2479,25 +2439,21 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Mickey Gasper</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>MIN</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>1</v>
-      </c>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>2026</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2512,25 +2468,21 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Jacob Lopez</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>NYM</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>1</v>
-      </c>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2545,25 +2497,21 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Kaelen Culpepper</t>
+          <t>Zach Thornton</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MIN</t>
-        </is>
-      </c>
-      <c r="E64" t="n">
-        <v>1</v>
-      </c>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2578,25 +2526,21 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Brandon Young</t>
+          <t>Zebby Matthews</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>BAL</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>1</v>
-      </c>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G65" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3997,24 +3941,24 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Dustin May</t>
+          <t>Joe Ryan</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="109">
@@ -4030,24 +3974,24 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Joe Ryan</t>
+          <t>Shane McClanahan</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="110">
@@ -4063,7 +4007,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Shane McClanahan</t>
+          <t>Drew Rasmussen</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -4072,7 +4016,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4096,16 +4040,16 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Drew Rasmussen</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -4129,12 +4073,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -4162,16 +4106,16 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -4195,12 +4139,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4228,16 +4172,16 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Jeff Hoffman</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -4261,20 +4205,20 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Jeff Hoffman</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -4294,20 +4238,20 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Brendan Donovan</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G117" t="n">
@@ -4327,24 +4271,24 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Brendan Donovan</t>
+          <t>Mason Miller</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G118" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="119">
@@ -4360,24 +4304,24 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Mason Miller</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="120">
@@ -4393,12 +4337,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Gerrit Cole</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4406,7 +4350,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G120" t="n">
@@ -4426,12 +4370,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Gerrit Cole</t>
+          <t>Jackson Jobe</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -4439,11 +4383,11 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G121" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="122">
@@ -4459,16 +4403,16 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Jackson Jobe</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -4492,16 +4436,16 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Cal Quantrill</t>
+          <t>Clay Holmes</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -4525,24 +4469,24 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Adrian Morejon</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G124" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="125">
@@ -4558,12 +4502,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Clay Holmes</t>
+          <t>Garrett Whitlock</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -4571,11 +4515,11 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="126">
@@ -4591,12 +4535,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Adrian Morejon</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4624,12 +4568,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Garrett Whitlock</t>
+          <t>Bryan Baker</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4637,11 +4581,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="128">
@@ -4657,12 +4601,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Bubba Chandler</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -4670,11 +4614,11 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G128" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="129">
@@ -4690,12 +4634,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Bryan Baker</t>
+          <t>Bryan Woo</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -4703,11 +4647,11 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="130">
@@ -4723,12 +4667,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Bubba Chandler</t>
+          <t>Franklin Arias</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -4736,7 +4680,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G130" t="n">
@@ -4756,25 +4700,21 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Heriberto Hernández</t>
+          <t>Cal Quantrill</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>MIA</t>
-        </is>
-      </c>
-      <c r="E131" t="n">
-        <v>1</v>
-      </c>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G131" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4789,25 +4729,21 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Kodai Senga</t>
+          <t>Dustin May</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>NYM</t>
-        </is>
-      </c>
-      <c r="E132" t="n">
-        <v>1</v>
-      </c>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G132" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4822,25 +4758,21 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Tim Tawa</t>
+          <t>Heriberto Hernández</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>ARI</t>
-        </is>
-      </c>
-      <c r="E133" t="n">
-        <v>1</v>
-      </c>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G133" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4855,25 +4787,21 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Kodai Senga</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>ATH</t>
-        </is>
-      </c>
-      <c r="E134" t="n">
-        <v>1</v>
-      </c>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G134" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4888,25 +4816,21 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Bryan Woo</t>
+          <t>Tim Tawa</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>SEA</t>
-        </is>
-      </c>
-      <c r="E135" t="n">
-        <v>1</v>
-      </c>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
-        </is>
-      </c>
-      <c r="G135" t="n">
-        <v>2026</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4921,25 +4845,21 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Franklin Arias</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>BOS</t>
-        </is>
-      </c>
-      <c r="E136" t="n">
-        <v>1</v>
-      </c>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G136" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -5944,12 +5864,12 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>Evan Phillips</t>
+          <t>Yusei Kikuchi</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E167" s="2" t="n">
@@ -5957,11 +5877,11 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G167" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="168">
@@ -5977,12 +5897,12 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Yusei Kikuchi</t>
+          <t>Joshua Baez</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E168" s="2" t="n">
@@ -5990,7 +5910,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G168" s="2" t="n">
@@ -6010,12 +5930,12 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>Joshua Baez</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E169" s="2" t="n">
@@ -6043,12 +5963,12 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E170" s="2" t="n">
@@ -6076,25 +5996,21 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Evan Phillips</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>CLE</t>
-        </is>
-      </c>
-      <c r="E171" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr"/>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G171" s="2" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6571,24 +6487,24 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Ryan Johnson</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G186" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="187">
@@ -6604,24 +6520,24 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Kyle Stowers</t>
+          <t>Tanner Scott</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G187" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="188">
@@ -6637,12 +6553,12 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Tanner Scott</t>
+          <t>Tyler Wells</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -6650,11 +6566,11 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G188" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="189">
@@ -6670,12 +6586,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Tyler Wells</t>
+          <t>Cade Smith</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -6683,7 +6599,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G189" t="n">
@@ -6703,12 +6619,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Cade Smith</t>
+          <t>Andrew Painter</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -6716,11 +6632,11 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G190" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="191">
@@ -6736,12 +6652,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Andrew Painter</t>
+          <t>River Ryan</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -6749,7 +6665,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G191" t="n">
@@ -6769,16 +6685,16 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>River Ryan</t>
+          <t>Anthony Volpe</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F192" t="inlineStr">
         <is>
@@ -6802,12 +6718,12 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Bryan Hudson</t>
+          <t>Louis Varland</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E193" t="n">
@@ -6835,12 +6751,12 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Luis Medina</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -6848,7 +6764,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G194" t="n">
@@ -6868,12 +6784,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Anthony Volpe</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E195" t="n">
@@ -6881,11 +6797,11 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G195" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="196">
@@ -6901,12 +6817,12 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Louis Varland</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E196" t="n">
@@ -6914,11 +6830,11 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G196" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="197">
@@ -6934,12 +6850,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Brent Headrick</t>
+          <t>Mason Montgomery</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E197" t="n">
@@ -6967,12 +6883,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Junior Caminero</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -6980,11 +6896,11 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G198" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="199">
@@ -7000,25 +6916,21 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Bryan Hudson</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>ATL</t>
-        </is>
-      </c>
-      <c r="E199" t="n">
-        <v>1</v>
-      </c>
+          <t>CWS</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
-        </is>
-      </c>
-      <c r="G199" t="n">
-        <v>2026</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -7033,25 +6945,21 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Luis Medina</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>CLE</t>
-        </is>
-      </c>
-      <c r="E200" t="n">
-        <v>1</v>
-      </c>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
-        </is>
-      </c>
-      <c r="G200" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -7066,7 +6974,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Brent Headrick</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -7074,17 +6982,13 @@
           <t>NYY</t>
         </is>
       </c>
-      <c r="E201" t="n">
-        <v>1</v>
-      </c>
+      <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G201" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -7099,25 +7003,21 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Mason Montgomery</t>
+          <t>Spencer Jones</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>PIT</t>
-        </is>
-      </c>
-      <c r="E202" t="n">
-        <v>1</v>
-      </c>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G202" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -7132,25 +7032,21 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Junior Caminero</t>
+          <t>Quinn Mathews</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>TB</t>
-        </is>
-      </c>
-      <c r="E203" t="n">
-        <v>1</v>
-      </c>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
-        </is>
-      </c>
-      <c r="G203" t="n">
-        <v>2026</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -7165,25 +7061,21 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Quinn Mathews</t>
+          <t>Ryan Johnson</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>STL</t>
-        </is>
-      </c>
-      <c r="E204" t="n">
-        <v>1</v>
-      </c>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G204" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -7206,17 +7098,13 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="E205" t="n">
-        <v>1</v>
-      </c>
+      <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G205" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -7759,16 +7647,16 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Kumar Rocker</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E222" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
@@ -7792,24 +7680,24 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Max Muncy</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E223" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G223" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="224">
@@ -7825,24 +7713,24 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Max Muncy</t>
+          <t>Peter Lambert</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="E224" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G224" s="2" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="225">
@@ -7858,12 +7746,12 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Peter Lambert</t>
+          <t>Merrill Kelly</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E225" s="2" t="n">
@@ -7871,11 +7759,11 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G225" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="226">
@@ -7891,12 +7779,12 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Merrill Kelly</t>
+          <t>Ryan Jeffers</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E226" s="2" t="n">
@@ -7904,7 +7792,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G226" s="2" t="n">
@@ -7924,12 +7812,12 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Ryan Jeffers</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E227" s="2" t="n">
@@ -7937,11 +7825,11 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G227" s="2" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="228">
@@ -7957,16 +7845,16 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Nick Martinez</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E228" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
@@ -7990,16 +7878,16 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>Nick Martinez</t>
+          <t>Eduardo Rodriguez</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E229" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
@@ -8023,24 +7911,24 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Robert Gasser</t>
+          <t>Matthew Liberatore</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E230" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="231">
@@ -8056,24 +7944,24 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E231" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (draft origin)</t>
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="232">
@@ -8089,12 +7977,12 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Eduardo Rodriguez</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E232" s="2" t="n">
@@ -8102,7 +7990,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G232" s="2" t="n">
@@ -8122,12 +8010,12 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Matthew Liberatore</t>
+          <t>Stephen Kolek</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E233" s="2" t="n">
@@ -8135,11 +8023,11 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G233" s="2" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="234">
@@ -8155,12 +8043,12 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Cole Carrigg</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E234" s="2" t="n">
@@ -8168,11 +8056,11 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>Kept — final year (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G234" s="2" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="235">
@@ -8188,7 +8076,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Zyhir Hope</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -8201,7 +8089,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G235" s="2" t="n">
@@ -8221,12 +8109,12 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Stephen Kolek</t>
+          <t>Chase Burns</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="E236" s="2" t="n">
@@ -8234,11 +8122,11 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — final year (waiver origin)</t>
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="237">
@@ -8254,25 +8142,21 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Robert Gasser</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>COL</t>
-        </is>
-      </c>
-      <c r="E237" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr"/>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G237" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -8287,25 +8171,21 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Zyhir Hope</t>
+          <t>Kumar Rocker</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
-        </is>
-      </c>
-      <c r="E238" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr"/>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G238" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -8320,25 +8200,21 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Chase Burns</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>CIN</t>
-        </is>
-      </c>
-      <c r="E239" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr"/>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>Kept — final year (waiver origin)</t>
-        </is>
-      </c>
-      <c r="G239" s="2" t="n">
-        <v>2026</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -8650,12 +8526,12 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E249" t="n">
@@ -8663,7 +8539,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — year 2 of 3 (pre-season waiver origin)</t>
         </is>
       </c>
       <c r="G249" t="n">
@@ -8683,12 +8559,12 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Ben Rice</t>
+          <t>Roki Sasaki</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E250" t="n">
@@ -8696,11 +8572,11 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (pre-season waiver origin)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G250" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="251">
@@ -8716,24 +8592,24 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Roki Sasaki</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G251" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="252">
@@ -8749,20 +8625,20 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Luis Severino</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G252" t="n">
@@ -8782,12 +8658,12 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Luis Severino</t>
+          <t>James Tibbs III</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E253" t="n">
@@ -8815,24 +8691,24 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Walker Buehler</t>
+          <t>Paul Sewald</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G254" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="255">
@@ -8848,16 +8724,16 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>James Tibbs III</t>
+          <t>Kody Clemens</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F255" t="inlineStr">
         <is>
@@ -8881,12 +8757,12 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Anthony Kay</t>
+          <t>Griffin Conine</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E256" t="n">
@@ -8914,12 +8790,12 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Paul Sewald</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E257" t="n">
@@ -8927,7 +8803,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G257" t="n">
@@ -8947,12 +8823,12 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Kody Clemens</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E258" t="n">
@@ -8960,11 +8836,11 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G258" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="259">
@@ -8980,12 +8856,12 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Cristian Javier</t>
+          <t>Sean Burke</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E259" t="n">
@@ -9013,12 +8889,12 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Taj Bradley</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E260" t="n">
@@ -9046,12 +8922,12 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Griffin Conine</t>
+          <t>Ian Seymour</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E261" t="n">
@@ -9059,11 +8935,11 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G261" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="262">
@@ -9079,12 +8955,12 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Miguel Vargas</t>
+          <t>Tristan Peters</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>CHW</t>
         </is>
       </c>
       <c r="E262" t="n">
@@ -9092,11 +8968,11 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G262" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="263">
@@ -9112,12 +8988,12 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Josue De Paula</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E263" t="n">
@@ -9125,7 +9001,7 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G263" t="n">
@@ -9145,12 +9021,12 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Sean Burke</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>CWS</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="E264" t="n">
@@ -9158,11 +9034,11 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G264" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="265">
@@ -9178,25 +9054,21 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Michael McGreevy</t>
+          <t>Walker Buehler</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>STL</t>
-        </is>
-      </c>
-      <c r="E265" t="n">
-        <v>1</v>
-      </c>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G265" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -9211,25 +9083,21 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Taj Bradley</t>
+          <t>Anthony Kay</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>MIN</t>
-        </is>
-      </c>
-      <c r="E266" t="n">
-        <v>1</v>
-      </c>
+          <t>CWS</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr"/>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G266" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -9244,25 +9112,21 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Ian Seymour</t>
+          <t>Cristian Javier</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>TB</t>
-        </is>
-      </c>
-      <c r="E267" t="n">
-        <v>1</v>
-      </c>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr"/>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G267" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -9277,25 +9141,21 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Tristan Peters</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>CHW</t>
-        </is>
-      </c>
-      <c r="E268" t="n">
-        <v>1</v>
-      </c>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr"/>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G268" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -9310,25 +9170,21 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Andrés Chaparro</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>WSH</t>
-        </is>
-      </c>
-      <c r="E269" t="n">
-        <v>1</v>
-      </c>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr"/>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G269" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -9343,25 +9199,21 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Didier Fuentes</t>
+          <t>Michael McGreevy</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>ATL</t>
-        </is>
-      </c>
-      <c r="E270" t="n">
-        <v>1</v>
-      </c>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr"/>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G270" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -9376,25 +9228,21 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Josue De Paula</t>
+          <t>Andrés Chaparro</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>LAD</t>
-        </is>
-      </c>
-      <c r="E271" t="n">
-        <v>1</v>
-      </c>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr"/>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G271" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -9409,25 +9257,21 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Mason Fluharty</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>HOU</t>
-        </is>
-      </c>
-      <c r="E272" t="n">
-        <v>1</v>
-      </c>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr"/>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G272" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -9442,18 +9286,18 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Mason Fluharty</t>
+          <t>Didier Fuentes</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E273" t="inlineStr"/>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Unknown (no acquisition record)</t>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
         </is>
       </c>
       <c r="G273" t="inlineStr"/>
@@ -10164,12 +10008,12 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>Tyler Mahle</t>
+          <t>Jakob Junis</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="E295" s="2" t="n">
@@ -10197,12 +10041,12 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>Jakob Junis</t>
+          <t>Jake Bauers</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E296" s="2" t="n">
@@ -10230,12 +10074,12 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>Jake Bauers</t>
+          <t>Andrés Giménez</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E297" s="2" t="n">
@@ -10243,11 +10087,11 @@
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="298">
@@ -10263,12 +10107,12 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Andrés Giménez</t>
+          <t>Casey Mize</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E298" s="2" t="n">
@@ -10296,12 +10140,12 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>Casey Mize</t>
+          <t>Kris Bubic</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E299" s="2" t="n">
@@ -10329,12 +10173,12 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Kris Bubic</t>
+          <t>Esteury Ruiz</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="E300" s="2" t="n">
@@ -10342,11 +10186,11 @@
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G300" s="2" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="301">
@@ -10362,12 +10206,12 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>Esteury Ruiz</t>
+          <t>Luis Campusano</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E301" s="2" t="n">
@@ -10395,12 +10239,12 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>Luis Campusano</t>
+          <t>Hogan Harris</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="E302" s="2" t="n">
@@ -10428,12 +10272,12 @@
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>Hogan Harris</t>
+          <t>Juan Morillo</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E303" s="2" t="n">
@@ -10461,12 +10305,12 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>Hao-Yu Lee</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E304" s="2" t="n">
@@ -10494,12 +10338,12 @@
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>Juan Morillo</t>
+          <t>Payton Tolle</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E305" s="2" t="n">
@@ -10507,11 +10351,11 @@
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G305" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="306">
@@ -10527,25 +10371,21 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Tyler Mahle</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>COL</t>
-        </is>
-      </c>
-      <c r="E306" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr"/>
       <c r="F306" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G306" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -10560,25 +10400,21 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>Abimelec Ortiz</t>
+          <t>Hao-Yu Lee</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>WSH</t>
-        </is>
-      </c>
-      <c r="E307" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr"/>
       <c r="F307" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G307" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G307" s="2" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
@@ -10593,25 +10429,21 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Payton Tolle</t>
+          <t>Abimelec Ortiz</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>BOS</t>
-        </is>
-      </c>
-      <c r="E308" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr"/>
       <c r="F308" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G308" s="2" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -12474,12 +12306,12 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>Andre Pallante</t>
+          <t>Ben Brown</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E365" s="2" t="n">
@@ -12487,11 +12319,11 @@
       </c>
       <c r="F365" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G365" s="2" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="366">
@@ -12507,12 +12339,12 @@
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>Ben Brown</t>
+          <t>Noah Cameron</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E366" s="2" t="n">
@@ -12520,7 +12352,7 @@
       </c>
       <c r="F366" s="2" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G366" s="2" t="n">
@@ -12540,12 +12372,12 @@
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>Noah Cameron</t>
+          <t>Kyle Leahy</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E367" s="2" t="n">
@@ -12553,11 +12385,11 @@
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G367" s="2" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="368">
@@ -12573,16 +12405,16 @@
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>Kyle Leahy</t>
+          <t>Taylor Clarke</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E368" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F368" s="2" t="inlineStr">
         <is>
@@ -12606,12 +12438,12 @@
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>Taylor Clarke</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E369" s="2" t="n">
@@ -12639,12 +12471,12 @@
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Samad Taylor</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>SDP</t>
         </is>
       </c>
       <c r="E370" s="2" t="n">
@@ -12672,12 +12504,12 @@
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>Samad Taylor</t>
+          <t>Victor Mesa Jr.</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E371" s="2" t="n">
@@ -12705,12 +12537,12 @@
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E372" s="2" t="n">
@@ -12738,25 +12570,21 @@
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>Victor Mesa Jr.</t>
+          <t>Andre Pallante</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
-        </is>
-      </c>
-      <c r="E373" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="E373" s="2" t="inlineStr"/>
       <c r="F373" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G373" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G373" s="2" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
@@ -12771,25 +12599,21 @@
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>SEA</t>
-        </is>
-      </c>
-      <c r="E374" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="inlineStr"/>
       <c r="F374" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G374" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G374" s="2" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
@@ -12812,17 +12636,13 @@
           <t>CHC</t>
         </is>
       </c>
-      <c r="E375" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="E375" s="2" t="inlineStr"/>
       <c r="F375" s="2" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
-        </is>
-      </c>
-      <c r="G375" s="2" t="n">
-        <v>2027</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G375" s="2" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -13266,12 +13086,12 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Max Scherzer</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E389" t="n">
@@ -13299,12 +13119,12 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E390" t="n">
@@ -13312,11 +13132,11 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G390" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="391">
@@ -13332,12 +13152,12 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Walbert Ureña</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E391" t="n">
@@ -13345,11 +13165,11 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G391" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="392">
@@ -13365,20 +13185,20 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Walbert Ureña</t>
+          <t>Trevor Story</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E392" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Kept — year 2 of 3 (draft origin)</t>
         </is>
       </c>
       <c r="G392" t="n">
@@ -13398,12 +13218,12 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Trevor Story</t>
+          <t>Alex Vesia</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E393" t="n">
@@ -13411,11 +13231,11 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Kept — year 2 of 3 (draft origin)</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G393" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="394">
@@ -13431,12 +13251,12 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Alex Vesia</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E394" t="n">
@@ -13444,7 +13264,7 @@
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G394" t="n">
@@ -13464,12 +13284,12 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Dillon Dingler</t>
+          <t>Orion Kerkering</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E395" t="n">
@@ -13477,7 +13297,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G395" t="n">
@@ -13497,20 +13317,20 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Orion Kerkering</t>
+          <t>Chris Bassitt</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E396" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G396" t="n">
@@ -13530,12 +13350,12 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Chris Bassitt</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E397" t="n">
@@ -13563,12 +13383,12 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Rico Garcia</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E398" t="n">
@@ -13576,11 +13396,11 @@
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G398" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="399">
@@ -13596,12 +13416,12 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Rico Garcia</t>
+          <t>Joey Cantillo</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E399" t="n">
@@ -13609,11 +13429,11 @@
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G399" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="400">
@@ -13629,12 +13449,12 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Joey Cantillo</t>
+          <t>Hayden Wesneski</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="E400" t="n">
@@ -13642,11 +13462,11 @@
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G400" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="401">
@@ -13662,12 +13482,12 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Hayden Wesneski</t>
+          <t>Jose A. Ferrer</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E401" t="n">
@@ -13675,11 +13495,11 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G401" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="402">
@@ -13695,12 +13515,12 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Jose A. Ferrer</t>
+          <t>Parker Messick</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E402" t="n">
@@ -13708,7 +13528,7 @@
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G402" t="n">
@@ -13728,12 +13548,12 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Parker Messick</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E403" t="n">
@@ -13741,7 +13561,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G403" t="n">
@@ -13761,12 +13581,12 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Will Warren</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E404" t="n">
@@ -13774,7 +13594,7 @@
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Drafted 2026 — year 1 of 3</t>
         </is>
       </c>
       <c r="G404" t="n">
@@ -13794,12 +13614,12 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Will Warren</t>
+          <t>Walker Jenkins</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E405" t="n">
@@ -13807,7 +13627,7 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Drafted 2026 — year 1 of 3</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G405" t="n">
@@ -13827,12 +13647,12 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Walker Jenkins</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>SFG</t>
         </is>
       </c>
       <c r="E406" t="n">
@@ -13860,12 +13680,12 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Pedro Ramirez</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E407" t="n">
@@ -13873,11 +13693,11 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
+          <t>Waiver — year 1 of 2</t>
         </is>
       </c>
       <c r="G407" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="408">
@@ -13893,12 +13713,12 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Pedro Ramirez</t>
+          <t>Jesús Made</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E408" t="n">
@@ -13906,11 +13726,11 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>Waiver — year 1 of 2</t>
+          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
         </is>
       </c>
       <c r="G408" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="409">
@@ -13926,25 +13746,21 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Jesús Made</t>
+          <t>Max Scherzer</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>MIL</t>
-        </is>
-      </c>
-      <c r="E409" t="n">
-        <v>1</v>
-      </c>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr"/>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Pre-season waiver — year 1 of 3 (drafted-equivalent)</t>
-        </is>
-      </c>
-      <c r="G409" t="n">
-        <v>2028</v>
-      </c>
+          <t>Waiver — added after the Aug 6 trade deadline; not keeper-eligible</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" s="3" t="inlineStr">

</xml_diff>